<commit_message>
code refactoring by claude
</commit_message>
<xml_diff>
--- a/public/Краткий отчет.xlsx
+++ b/public/Краткий отчет.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6819" uniqueCount="5582">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6936" uniqueCount="5661">
   <si>
     <t>Краткий отчет по товарам</t>
   </si>
@@ -16760,6 +16760,243 @@
   </si>
   <si>
     <t>Пододеяльник страйп-сатин 150х200 - М - 135 - Бежевый крем 1х1</t>
+  </si>
+  <si>
+    <t>4660674648159</t>
+  </si>
+  <si>
+    <t>Простыня микросатин 240х260 - "Бездна"</t>
+  </si>
+  <si>
+    <t>26-03-2026</t>
+  </si>
+  <si>
+    <t>4660674648142</t>
+  </si>
+  <si>
+    <t>КПБ Постельное бельё тенсель 1,5 спальное - "Песочная роза" наволочки 50х70</t>
+  </si>
+  <si>
+    <t>4660674648135</t>
+  </si>
+  <si>
+    <t>Пододеяльник бязь 145х215 - М - 120 - Музыкальные Совята</t>
+  </si>
+  <si>
+    <t>4660674648128</t>
+  </si>
+  <si>
+    <t>Пододеяльник бязь 145х215 - М - 120 - Розовый Воздух</t>
+  </si>
+  <si>
+    <t>4660674648111</t>
+  </si>
+  <si>
+    <t>Пододеяльник микрофибра 175х215 - "Петкана"</t>
+  </si>
+  <si>
+    <t>4610594539990</t>
+  </si>
+  <si>
+    <t>Наволочка сатин-твил 50х70 - "Фиорелла"</t>
+  </si>
+  <si>
+    <t>4610594539983</t>
+  </si>
+  <si>
+    <t>Простыня полисатин резинка 120х200х30 - "Мелиссит"</t>
+  </si>
+  <si>
+    <t>4610594539976</t>
+  </si>
+  <si>
+    <t>Пододеяльник сатин твил 175х215 - "Фиорелла"</t>
+  </si>
+  <si>
+    <t>4610594539969</t>
+  </si>
+  <si>
+    <t>Пододеяльник полисатин 220х240 - "Зайга"</t>
+  </si>
+  <si>
+    <t>4610594539952</t>
+  </si>
+  <si>
+    <t>Пододеяльник сатин 175х215 - "Агапия"</t>
+  </si>
+  <si>
+    <t>4610594539945</t>
+  </si>
+  <si>
+    <t>КПБ Постельное бельё бязь 2 спальное резинка 140х200х30 - "Пухлянки"</t>
+  </si>
+  <si>
+    <t>4610594539938</t>
+  </si>
+  <si>
+    <t>КПБ Постельное бельё сатин твил Евро - "Фернанда"</t>
+  </si>
+  <si>
+    <t>4610594539921</t>
+  </si>
+  <si>
+    <t>Наволочка поплин 50х50 - Гранола</t>
+  </si>
+  <si>
+    <t>4610594539914</t>
+  </si>
+  <si>
+    <t>КПБ Постельное бельё поплин Евро резинка 160х200х30 - "Глария"</t>
+  </si>
+  <si>
+    <t>4610594539907</t>
+  </si>
+  <si>
+    <t>Наволочка сатин 50х70 - Премиум ТС 320 Вишенка</t>
+  </si>
+  <si>
+    <t>4610594539891</t>
+  </si>
+  <si>
+    <t>Простыня сатин 200х220 - Премиум ТС 320 Бесконечность</t>
+  </si>
+  <si>
+    <t>4610594539884</t>
+  </si>
+  <si>
+    <t>Пододеяльник сатин 175х215 - М - Премиум ТС 320 Бесконечность</t>
+  </si>
+  <si>
+    <t>4610594539877</t>
+  </si>
+  <si>
+    <t>Простыня тенсель резинка 180х200х30 - Розовая лаванда</t>
+  </si>
+  <si>
+    <t>4610594539860</t>
+  </si>
+  <si>
+    <t>Простыня полисатин 260х260 - "Глубь"</t>
+  </si>
+  <si>
+    <t>4610594539853</t>
+  </si>
+  <si>
+    <t>Простыня сатин твил 260х260 - "Сахарная роза"</t>
+  </si>
+  <si>
+    <t>4610594539846</t>
+  </si>
+  <si>
+    <t>Наволочка тенсель 50х70 - "Твист"</t>
+  </si>
+  <si>
+    <t>4610594539839</t>
+  </si>
+  <si>
+    <t>Наволочка тенсель 70х70 - "Небра"</t>
+  </si>
+  <si>
+    <t>4610594539822</t>
+  </si>
+  <si>
+    <t>Простыня страйп-поплин 200 х 220 - М - Гестхаус Белый 3х3</t>
+  </si>
+  <si>
+    <t>4610594539815</t>
+  </si>
+  <si>
+    <t>Простыня варёный хлопок 240х260 - 323 Серый</t>
+  </si>
+  <si>
+    <t>4610594539808</t>
+  </si>
+  <si>
+    <t>Простыня перкаль резинка 200х220х20 - "Чёрное масло"</t>
+  </si>
+  <si>
+    <t>4610594539792</t>
+  </si>
+  <si>
+    <t>КПБ Постельное бельё микрофибра 1,5 спальное резинка 120х200х30 - "Альбелла" 1х1 наволочки 50х70</t>
+  </si>
+  <si>
+    <t>4610594539785</t>
+  </si>
+  <si>
+    <t>КПБ Постельное бельё тенсель 2 спальное - "Коньячный" наволочки 50х70</t>
+  </si>
+  <si>
+    <t>4610594539778</t>
+  </si>
+  <si>
+    <t>Простыня тенсель 260х260 - Чериньола</t>
+  </si>
+  <si>
+    <t>4610594539761</t>
+  </si>
+  <si>
+    <t>КПБ Постельное бельё тенсель 1,5 спальное резинка 90х200х30 - 41-020 Серебряный наволочки 50х70</t>
+  </si>
+  <si>
+    <t>4610594539754</t>
+  </si>
+  <si>
+    <t>КПБ Постельное бельё сатин твил 1,5 спальное резинка 120х200х30 - "Дино-пати" наволочки 50х70</t>
+  </si>
+  <si>
+    <t>4610594539747</t>
+  </si>
+  <si>
+    <t>Наволочка сатин 70х70 - 125 - Тёплый песок</t>
+  </si>
+  <si>
+    <t>4610594539730</t>
+  </si>
+  <si>
+    <t>Простыня бязь 80х120 - 142 ГОСТ - Темно-синяя</t>
+  </si>
+  <si>
+    <t>4610594539723</t>
+  </si>
+  <si>
+    <t>Простыня сатин твил 300х300 - "Лебединое перо"</t>
+  </si>
+  <si>
+    <t>4610594539716</t>
+  </si>
+  <si>
+    <t>Простыня полисатин 300х300 - "Олуфими"</t>
+  </si>
+  <si>
+    <t>4610594539709</t>
+  </si>
+  <si>
+    <t>Простыня страйп-сатин 300х300 - 135 - Платина 1х1</t>
+  </si>
+  <si>
+    <t>4610594539693</t>
+  </si>
+  <si>
+    <t>Простыня круглая микросатин резинка 200х200х20 - "Смоки"</t>
+  </si>
+  <si>
+    <t>4610594539686</t>
+  </si>
+  <si>
+    <t>КПБ Постельное бельё варёный хлопок 2 спальное резинка 140х200х30 - Бертолеция наволочки 50х70</t>
+  </si>
+  <si>
+    <t>4610594539679</t>
+  </si>
+  <si>
+    <t>Пододеяльник поплин 200х220 - "Сирента"</t>
+  </si>
+  <si>
+    <t>4610594539662</t>
+  </si>
+  <si>
+    <t>КПБ Постельное бельё тенсель 2 спальное резинка 160х200х30 - "Морозный туман"</t>
   </si>
 </sst>
 </file>
@@ -43146,6 +43383,435 @@
         <v>5465</v>
       </c>
     </row>
+    <row r="2776" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2776" t="s">
+        <v>5582</v>
+      </c>
+      <c r="B2776" t="s">
+        <v>5583</v>
+      </c>
+      <c r="C2776" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2777" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2777" t="s">
+        <v>5585</v>
+      </c>
+      <c r="B2777" t="s">
+        <v>5586</v>
+      </c>
+      <c r="C2777" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2778" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2778" t="s">
+        <v>5587</v>
+      </c>
+      <c r="B2778" t="s">
+        <v>5588</v>
+      </c>
+      <c r="C2778" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2779" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2779" t="s">
+        <v>5589</v>
+      </c>
+      <c r="B2779" t="s">
+        <v>5590</v>
+      </c>
+      <c r="C2779" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2780" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2780" t="s">
+        <v>5591</v>
+      </c>
+      <c r="B2780" t="s">
+        <v>5592</v>
+      </c>
+      <c r="C2780" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2781" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2781" t="s">
+        <v>5593</v>
+      </c>
+      <c r="B2781" t="s">
+        <v>5594</v>
+      </c>
+      <c r="C2781" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2782" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2782" t="s">
+        <v>5595</v>
+      </c>
+      <c r="B2782" t="s">
+        <v>5596</v>
+      </c>
+      <c r="C2782" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2783" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2783" t="s">
+        <v>5597</v>
+      </c>
+      <c r="B2783" t="s">
+        <v>5598</v>
+      </c>
+      <c r="C2783" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2784" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2784" t="s">
+        <v>5599</v>
+      </c>
+      <c r="B2784" t="s">
+        <v>5600</v>
+      </c>
+      <c r="C2784" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2785" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2785" t="s">
+        <v>5601</v>
+      </c>
+      <c r="B2785" t="s">
+        <v>5602</v>
+      </c>
+      <c r="C2785" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2786" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2786" t="s">
+        <v>5603</v>
+      </c>
+      <c r="B2786" t="s">
+        <v>5604</v>
+      </c>
+      <c r="C2786" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2787" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2787" t="s">
+        <v>5605</v>
+      </c>
+      <c r="B2787" t="s">
+        <v>5606</v>
+      </c>
+      <c r="C2787" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2788" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2788" t="s">
+        <v>5607</v>
+      </c>
+      <c r="B2788" t="s">
+        <v>5608</v>
+      </c>
+      <c r="C2788" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2789" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2789" t="s">
+        <v>5609</v>
+      </c>
+      <c r="B2789" t="s">
+        <v>5610</v>
+      </c>
+      <c r="C2789" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2790" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2790" t="s">
+        <v>5611</v>
+      </c>
+      <c r="B2790" t="s">
+        <v>5612</v>
+      </c>
+      <c r="C2790" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2791" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2791" t="s">
+        <v>5613</v>
+      </c>
+      <c r="B2791" t="s">
+        <v>5614</v>
+      </c>
+      <c r="C2791" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2792" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2792" t="s">
+        <v>5615</v>
+      </c>
+      <c r="B2792" t="s">
+        <v>5616</v>
+      </c>
+      <c r="C2792" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2793" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2793" t="s">
+        <v>5617</v>
+      </c>
+      <c r="B2793" t="s">
+        <v>5618</v>
+      </c>
+      <c r="C2793" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2794" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2794" t="s">
+        <v>5619</v>
+      </c>
+      <c r="B2794" t="s">
+        <v>5620</v>
+      </c>
+      <c r="C2794" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2795" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2795" t="s">
+        <v>5621</v>
+      </c>
+      <c r="B2795" t="s">
+        <v>5622</v>
+      </c>
+      <c r="C2795" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2796" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2796" t="s">
+        <v>5623</v>
+      </c>
+      <c r="B2796" t="s">
+        <v>5624</v>
+      </c>
+      <c r="C2796" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2797" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2797" t="s">
+        <v>5625</v>
+      </c>
+      <c r="B2797" t="s">
+        <v>5626</v>
+      </c>
+      <c r="C2797" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2798" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2798" t="s">
+        <v>5627</v>
+      </c>
+      <c r="B2798" t="s">
+        <v>5628</v>
+      </c>
+      <c r="C2798" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2799" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2799" t="s">
+        <v>5629</v>
+      </c>
+      <c r="B2799" t="s">
+        <v>5630</v>
+      </c>
+      <c r="C2799" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2800" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2800" t="s">
+        <v>5631</v>
+      </c>
+      <c r="B2800" t="s">
+        <v>5632</v>
+      </c>
+      <c r="C2800" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2801" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2801" t="s">
+        <v>5633</v>
+      </c>
+      <c r="B2801" t="s">
+        <v>5634</v>
+      </c>
+      <c r="C2801" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2802" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2802" t="s">
+        <v>5635</v>
+      </c>
+      <c r="B2802" t="s">
+        <v>5636</v>
+      </c>
+      <c r="C2802" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2803" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2803" t="s">
+        <v>5637</v>
+      </c>
+      <c r="B2803" t="s">
+        <v>5638</v>
+      </c>
+      <c r="C2803" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2804" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2804" t="s">
+        <v>5639</v>
+      </c>
+      <c r="B2804" t="s">
+        <v>5640</v>
+      </c>
+      <c r="C2804" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2805" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2805" t="s">
+        <v>5641</v>
+      </c>
+      <c r="B2805" t="s">
+        <v>5642</v>
+      </c>
+      <c r="C2805" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2806" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2806" t="s">
+        <v>5643</v>
+      </c>
+      <c r="B2806" t="s">
+        <v>5644</v>
+      </c>
+      <c r="C2806" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2807" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2807" t="s">
+        <v>5645</v>
+      </c>
+      <c r="B2807" t="s">
+        <v>5646</v>
+      </c>
+      <c r="C2807" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2808" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2808" t="s">
+        <v>5647</v>
+      </c>
+      <c r="B2808" t="s">
+        <v>5648</v>
+      </c>
+      <c r="C2808" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2809" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2809" t="s">
+        <v>5649</v>
+      </c>
+      <c r="B2809" t="s">
+        <v>5650</v>
+      </c>
+      <c r="C2809" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2810" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2810" t="s">
+        <v>5651</v>
+      </c>
+      <c r="B2810" t="s">
+        <v>5652</v>
+      </c>
+      <c r="C2810" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2811" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2811" t="s">
+        <v>5653</v>
+      </c>
+      <c r="B2811" t="s">
+        <v>5654</v>
+      </c>
+      <c r="C2811" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2812" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2812" t="s">
+        <v>5655</v>
+      </c>
+      <c r="B2812" t="s">
+        <v>5656</v>
+      </c>
+      <c r="C2812" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2813" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2813" t="s">
+        <v>5657</v>
+      </c>
+      <c r="B2813" t="s">
+        <v>5658</v>
+      </c>
+      <c r="C2813" t="s">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="2814" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2814" t="s">
+        <v>5659</v>
+      </c>
+      <c r="B2814" t="s">
+        <v>5660</v>
+      </c>
+      <c r="C2814" t="s">
+        <v>5584</v>
+      </c>
+    </row>
     <row r="3449" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3449" s="6"/>
     </row>

</xml_diff>

<commit_message>
update short report & actual.html
</commit_message>
<xml_diff>
--- a/public/Краткий отчет.xlsx
+++ b/public/Краткий отчет.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7221" uniqueCount="5853">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7254" uniqueCount="5876">
   <si>
     <t>Краткий отчет по товарам</t>
   </si>
@@ -17573,6 +17573,75 @@
   </si>
   <si>
     <t>КПБ Постельное бельё жатка 1,5 спальное резинка 120х200х30 - "Звёздный Вальс" наволочки 50х70</t>
+  </si>
+  <si>
+    <t>4660674649217</t>
+  </si>
+  <si>
+    <t>Наволочка сатин браш 50х70 - Кремовый бархат</t>
+  </si>
+  <si>
+    <t>31-03-2026</t>
+  </si>
+  <si>
+    <t>4660674649200</t>
+  </si>
+  <si>
+    <t>Простыня тенсель резинка 140х200х30 - "Карибская волна"</t>
+  </si>
+  <si>
+    <t>4660674649194</t>
+  </si>
+  <si>
+    <t>Пододеяльник микросатин 150х200 - "Страстный гранат"</t>
+  </si>
+  <si>
+    <t>4660674649187</t>
+  </si>
+  <si>
+    <t>Простыня полисатин 260х260 - "Гуголету"</t>
+  </si>
+  <si>
+    <t>4660674649170</t>
+  </si>
+  <si>
+    <t>Простыня варёный хлопок резинка 140х200х30 - Белый</t>
+  </si>
+  <si>
+    <t>4660674649163</t>
+  </si>
+  <si>
+    <t>КПБ Постельное бельё тенсель King Size семейное резинка 200х200х30 - 74 Оливковый</t>
+  </si>
+  <si>
+    <t>4660674649156</t>
+  </si>
+  <si>
+    <t>КПБ Постельное бельё тенсель семейное резинка 180х200х30 - Прохлада ментола наволочки 50х70</t>
+  </si>
+  <si>
+    <t>4660674649149</t>
+  </si>
+  <si>
+    <t>Наволочка тенсель 40х60 - "Дюна"</t>
+  </si>
+  <si>
+    <t>4660674649132</t>
+  </si>
+  <si>
+    <t>Простыня страйп-сатин резинка 180х200х45 - 130 - "Лучезарный" 1х1</t>
+  </si>
+  <si>
+    <t>4660674649125</t>
+  </si>
+  <si>
+    <t>КПБ Постельное бельё тенсель семейное резинка 160х200х30 - "Бейж"</t>
+  </si>
+  <si>
+    <t>4660674649118</t>
+  </si>
+  <si>
+    <t>Пододеяльник страйп-сатин 200х200 - М - 140 - Миндаль 1х1</t>
   </si>
 </sst>
 </file>
@@ -45433,6 +45502,127 @@
         <v>5732</v>
       </c>
     </row>
+    <row r="2910" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2910" t="s">
+        <v>5853</v>
+      </c>
+      <c r="B2910" t="s">
+        <v>5854</v>
+      </c>
+      <c r="C2910" t="s">
+        <v>5855</v>
+      </c>
+    </row>
+    <row r="2911" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2911" t="s">
+        <v>5856</v>
+      </c>
+      <c r="B2911" t="s">
+        <v>5857</v>
+      </c>
+      <c r="C2911" t="s">
+        <v>5855</v>
+      </c>
+    </row>
+    <row r="2912" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2912" t="s">
+        <v>5858</v>
+      </c>
+      <c r="B2912" t="s">
+        <v>5859</v>
+      </c>
+      <c r="C2912" t="s">
+        <v>5855</v>
+      </c>
+    </row>
+    <row r="2913" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2913" t="s">
+        <v>5860</v>
+      </c>
+      <c r="B2913" t="s">
+        <v>5861</v>
+      </c>
+      <c r="C2913" t="s">
+        <v>5855</v>
+      </c>
+    </row>
+    <row r="2914" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2914" t="s">
+        <v>5862</v>
+      </c>
+      <c r="B2914" t="s">
+        <v>5863</v>
+      </c>
+      <c r="C2914" t="s">
+        <v>5855</v>
+      </c>
+    </row>
+    <row r="2915" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2915" t="s">
+        <v>5864</v>
+      </c>
+      <c r="B2915" t="s">
+        <v>5865</v>
+      </c>
+      <c r="C2915" t="s">
+        <v>5855</v>
+      </c>
+    </row>
+    <row r="2916" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2916" t="s">
+        <v>5866</v>
+      </c>
+      <c r="B2916" t="s">
+        <v>5867</v>
+      </c>
+      <c r="C2916" t="s">
+        <v>5855</v>
+      </c>
+    </row>
+    <row r="2917" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2917" t="s">
+        <v>5868</v>
+      </c>
+      <c r="B2917" t="s">
+        <v>5869</v>
+      </c>
+      <c r="C2917" t="s">
+        <v>5855</v>
+      </c>
+    </row>
+    <row r="2918" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2918" t="s">
+        <v>5870</v>
+      </c>
+      <c r="B2918" t="s">
+        <v>5871</v>
+      </c>
+      <c r="C2918" t="s">
+        <v>5855</v>
+      </c>
+    </row>
+    <row r="2919" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2919" t="s">
+        <v>5872</v>
+      </c>
+      <c r="B2919" t="s">
+        <v>5873</v>
+      </c>
+      <c r="C2919" t="s">
+        <v>5855</v>
+      </c>
+    </row>
+    <row r="2920" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2920" t="s">
+        <v>5874</v>
+      </c>
+      <c r="B2920" t="s">
+        <v>5875</v>
+      </c>
+      <c r="C2920" t="s">
+        <v>5855</v>
+      </c>
+    </row>
     <row r="3449" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3449" s="6"/>
     </row>

</xml_diff>